<commit_message>
test: add student activity logs tests
</commit_message>
<xml_diff>
--- a/scr/uploads/Students.xlsx
+++ b/scr/uploads/Students.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,392 +437,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TCC00021</v>
+        <v>TCC00001</v>
       </c>
       <c r="B2" t="str">
-        <v>Lade</v>
+        <v>John</v>
       </c>
       <c r="C2" t="str">
-        <v>Ololade</v>
+        <v>Doe</v>
       </c>
       <c r="D2" t="str">
-        <v>ooo</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="F2" s="1">
-        <v>40252.04207175926</v>
+        <v>41039.04207175926</v>
       </c>
       <c r="G2" t="str">
-        <v>JSS2</v>
+        <v>JSS1</v>
       </c>
       <c r="H2" t="str">
         <v>2025/2026</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Mr Doe</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>08011111111</v>
       </c>
       <c r="K2" s="1">
-        <v>46233.7439772338</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>TCC00020</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Lade</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Tioluwa</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>Female</v>
-      </c>
-      <c r="F3" s="1">
-        <v>41713.04207175926</v>
-      </c>
-      <c r="G3" t="str">
-        <v>JSS3</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2025/2026</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" s="1">
-        <v>46233.72479988426</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>TCC00019</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Peter</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Johnson</v>
-      </c>
-      <c r="D4" t="str">
-        <v>James</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F4" s="1">
-        <v>40852.04207175926</v>
-      </c>
-      <c r="G4" t="str">
-        <v>SS1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Mr Johnson</v>
-      </c>
-      <c r="J4" t="str">
-        <v>08011223344</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46233.63410418981</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>TCC00018</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Jane</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Smith</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v>Female</v>
-      </c>
-      <c r="F5" s="1">
-        <v>41475.04207175926</v>
-      </c>
-      <c r="G5" t="str">
-        <v>JSS2</v>
-      </c>
-      <c r="H5" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Mrs Smith</v>
-      </c>
-      <c r="J5" t="str">
-        <v>08087654321</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46233.63409685185</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>TCC00017</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Pjazz</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F6" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G6" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H6" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" s="1">
-        <v>46233.517736898146</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>TCC00016</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Pjazz</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F7" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G7" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H7" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" s="1">
-        <v>46233.51763679398</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>TCC00015</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Pjazz</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F8" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G8" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H8" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8" s="1">
-        <v>46233.51753513889</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>TCC00014</v>
-      </c>
-      <c r="B9" t="str">
-        <v>John</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F9" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G9" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H9" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9" s="1">
-        <v>46233.48381790509</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>TCC00013</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Faith</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Moses</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Michael</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Female</v>
-      </c>
-      <c r="F10" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G10" t="str">
-        <v>JSS3</v>
-      </c>
-      <c r="H10" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I10" t="str">
-        <v>Mr Moses</v>
-      </c>
-      <c r="J10" t="str">
-        <v>08012345678</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46232.96236806713</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>TCC00012</v>
-      </c>
-      <c r="B11" t="str">
-        <v>John</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Michael</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F11" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G11" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H11" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I11" t="str">
-        <v>Mr Doe</v>
-      </c>
-      <c r="J11" t="str">
-        <v>08012345678</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46232.96101503472</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>TCC00001</v>
-      </c>
-      <c r="B12" t="str">
-        <v>John</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Doe</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Michael</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Male</v>
-      </c>
-      <c r="F12" s="1">
-        <v>40983.04207175926</v>
-      </c>
-      <c r="G12" t="str">
-        <v>JSS1</v>
-      </c>
-      <c r="H12" t="str">
-        <v>2026/2027</v>
-      </c>
-      <c r="I12" t="str">
-        <v>Mr Doe</v>
-      </c>
-      <c r="J12" t="str">
-        <v>08012345678</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46231.93995008102</v>
+        <v>46245.872525844905</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>